<commit_message>
fix: close recommendation approval gate residuals
</commit_message>
<xml_diff>
--- a/docs/reviews/Sookta_Recommendation_Translation_Review_2026-07-29.xlsx
+++ b/docs/reviews/Sookta_Recommendation_Translation_Review_2026-07-29.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Review" sheetId="1" r:id="Rb71f2d3556e44bbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="Rbbf2ae8a147540dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="R04c7ed3e95044a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="4" r:id="R1c27fc88fc9b4634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="5" r:id="R532d5d6785634283"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="6" r:id="R745d4ed2d6854190"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R155f65f36fc5434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Review" sheetId="1" r:id="R923c13babebb49bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Catalog" sheetId="2" r:id="Ra634adb2e52c4f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="R1a02e03b9e7e46ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conflicts" sheetId="4" r:id="Re6837300329e4c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="5" r:id="Ra16effaccdc44775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="6" r:id="R08fff079f4884336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R102b4baebaa74bf8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,14 +401,15 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GateAuditTable" displayName="GateAuditTable" ref="A1:E176" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:E176"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GateAuditTable" displayName="GateAuditTable" ref="A1:F176" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F176"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="recommendation_id"/>
     <x:tableColumn id="2" name="english_contains_thai"/>
     <x:tableColumn id="3" name="invalid_translation_style"/>
     <x:tableColumn id="4" name="invalid_approved_at"/>
     <x:tableColumn id="5" name="invalid_translation_version"/>
+    <x:tableColumn id="6" name="invalid_units_not_applicable"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -10664,7 +10665,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57ef3d783069403d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c036ba39db3438a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20136,7 +20137,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R221eed99b65142bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2719a6b87c5e456e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20340,7 +20341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8caeedd1fb9949fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97eca2ced0a642ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20529,7 +20530,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R076200c134c547a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29d8af9f6de64b77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20543,6 +20544,7 @@
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -20561,6 +20563,9 @@
       <x:c r="E1" s="7" t="str">
         <x:v>invalid_translation_version</x:v>
       </x:c>
+      <x:c r="F1" s="7" t="str">
+        <x:v>invalid_units_not_applicable</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -20582,6 +20587,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q2),'Translation Review'!Q2&gt;0,'Translation Review'!Q2=INT('Translation Review'!Q2)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F2" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H2="not_applicable",IFERROR(REGEXTEST('Translation Review'!D2,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="8" t="str">
@@ -20603,6 +20612,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q3),'Translation Review'!Q3&gt;0,'Translation Review'!Q3=INT('Translation Review'!Q3)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F3" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H3="not_applicable",IFERROR(REGEXTEST('Translation Review'!D3,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -20624,6 +20637,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q4),'Translation Review'!Q4&gt;0,'Translation Review'!Q4=INT('Translation Review'!Q4)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F4" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H4="not_applicable",IFERROR(REGEXTEST('Translation Review'!D4,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="8" t="str">
@@ -20645,6 +20662,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q5),'Translation Review'!Q5&gt;0,'Translation Review'!Q5=INT('Translation Review'!Q5)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F5" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H5="not_applicable",IFERROR(REGEXTEST('Translation Review'!D5,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="8" t="str">
@@ -20666,6 +20687,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q6),'Translation Review'!Q6&gt;0,'Translation Review'!Q6=INT('Translation Review'!Q6)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F6" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H6="not_applicable",IFERROR(REGEXTEST('Translation Review'!D6,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -20687,6 +20712,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q7),'Translation Review'!Q7&gt;0,'Translation Review'!Q7=INT('Translation Review'!Q7)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F7" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H7="not_applicable",IFERROR(REGEXTEST('Translation Review'!D7,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="8" t="str">
@@ -20708,6 +20737,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q8),'Translation Review'!Q8&gt;0,'Translation Review'!Q8=INT('Translation Review'!Q8)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F8" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H8="not_applicable",IFERROR(REGEXTEST('Translation Review'!D8,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="8" t="str">
@@ -20729,6 +20762,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q9),'Translation Review'!Q9&gt;0,'Translation Review'!Q9=INT('Translation Review'!Q9)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F9" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H9="not_applicable",IFERROR(REGEXTEST('Translation Review'!D9,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="8" t="str">
@@ -20750,6 +20787,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q10),'Translation Review'!Q10&gt;0,'Translation Review'!Q10=INT('Translation Review'!Q10)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F10" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H10="not_applicable",IFERROR(REGEXTEST('Translation Review'!D10,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="8" t="str">
@@ -20771,6 +20812,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q11),'Translation Review'!Q11&gt;0,'Translation Review'!Q11=INT('Translation Review'!Q11)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F11" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H11="not_applicable",IFERROR(REGEXTEST('Translation Review'!D11,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="8" t="str">
@@ -20792,6 +20837,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q12),'Translation Review'!Q12&gt;0,'Translation Review'!Q12=INT('Translation Review'!Q12)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F12" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H12="not_applicable",IFERROR(REGEXTEST('Translation Review'!D12,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="8" t="str">
@@ -20813,6 +20862,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q13),'Translation Review'!Q13&gt;0,'Translation Review'!Q13=INT('Translation Review'!Q13)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F13" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H13="not_applicable",IFERROR(REGEXTEST('Translation Review'!D13,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="8" t="str">
@@ -20834,6 +20887,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q14),'Translation Review'!Q14&gt;0,'Translation Review'!Q14=INT('Translation Review'!Q14)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F14" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H14="not_applicable",IFERROR(REGEXTEST('Translation Review'!D14,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="8" t="str">
@@ -20855,6 +20912,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q15),'Translation Review'!Q15&gt;0,'Translation Review'!Q15=INT('Translation Review'!Q15)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F15" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H15="not_applicable",IFERROR(REGEXTEST('Translation Review'!D15,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="8" t="str">
@@ -20876,6 +20937,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q16),'Translation Review'!Q16&gt;0,'Translation Review'!Q16=INT('Translation Review'!Q16)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F16" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H16="not_applicable",IFERROR(REGEXTEST('Translation Review'!D16,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="8" t="str">
@@ -20897,6 +20962,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q17),'Translation Review'!Q17&gt;0,'Translation Review'!Q17=INT('Translation Review'!Q17)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F17" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H17="not_applicable",IFERROR(REGEXTEST('Translation Review'!D17,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="8" t="str">
@@ -20918,6 +20987,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q18),'Translation Review'!Q18&gt;0,'Translation Review'!Q18=INT('Translation Review'!Q18)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F18" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H18="not_applicable",IFERROR(REGEXTEST('Translation Review'!D18,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="8" t="str">
@@ -20939,6 +21012,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q19),'Translation Review'!Q19&gt;0,'Translation Review'!Q19=INT('Translation Review'!Q19)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F19" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H19="not_applicable",IFERROR(REGEXTEST('Translation Review'!D19,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="8" t="str">
@@ -20960,6 +21037,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q20),'Translation Review'!Q20&gt;0,'Translation Review'!Q20=INT('Translation Review'!Q20)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F20" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H20="not_applicable",IFERROR(REGEXTEST('Translation Review'!D20,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="8" t="str">
@@ -20981,6 +21062,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q21),'Translation Review'!Q21&gt;0,'Translation Review'!Q21=INT('Translation Review'!Q21)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F21" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H21="not_applicable",IFERROR(REGEXTEST('Translation Review'!D21,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="8" t="str">
@@ -21002,6 +21087,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q22),'Translation Review'!Q22&gt;0,'Translation Review'!Q22=INT('Translation Review'!Q22)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F22" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H22="not_applicable",IFERROR(REGEXTEST('Translation Review'!D22,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="8" t="str">
@@ -21023,6 +21112,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q23),'Translation Review'!Q23&gt;0,'Translation Review'!Q23=INT('Translation Review'!Q23)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F23" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H23="not_applicable",IFERROR(REGEXTEST('Translation Review'!D23,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="8" t="str">
@@ -21044,6 +21137,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q24),'Translation Review'!Q24&gt;0,'Translation Review'!Q24=INT('Translation Review'!Q24)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F24" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H24="not_applicable",IFERROR(REGEXTEST('Translation Review'!D24,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="8" t="str">
@@ -21065,6 +21162,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q25),'Translation Review'!Q25&gt;0,'Translation Review'!Q25=INT('Translation Review'!Q25)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F25" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H25="not_applicable",IFERROR(REGEXTEST('Translation Review'!D25,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="8" t="str">
@@ -21086,6 +21187,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q26),'Translation Review'!Q26&gt;0,'Translation Review'!Q26=INT('Translation Review'!Q26)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F26" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H26="not_applicable",IFERROR(REGEXTEST('Translation Review'!D26,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="8" t="str">
@@ -21107,6 +21212,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q27),'Translation Review'!Q27&gt;0,'Translation Review'!Q27=INT('Translation Review'!Q27)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F27" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H27="not_applicable",IFERROR(REGEXTEST('Translation Review'!D27,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="8" t="str">
@@ -21128,6 +21237,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q28),'Translation Review'!Q28&gt;0,'Translation Review'!Q28=INT('Translation Review'!Q28)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F28" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H28="not_applicable",IFERROR(REGEXTEST('Translation Review'!D28,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="8" t="str">
@@ -21149,6 +21262,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q29),'Translation Review'!Q29&gt;0,'Translation Review'!Q29=INT('Translation Review'!Q29)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F29" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H29="not_applicable",IFERROR(REGEXTEST('Translation Review'!D29,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="8" t="str">
@@ -21170,6 +21287,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q30),'Translation Review'!Q30&gt;0,'Translation Review'!Q30=INT('Translation Review'!Q30)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F30" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H30="not_applicable",IFERROR(REGEXTEST('Translation Review'!D30,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="8" t="str">
@@ -21191,6 +21312,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q31),'Translation Review'!Q31&gt;0,'Translation Review'!Q31=INT('Translation Review'!Q31)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F31" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H31="not_applicable",IFERROR(REGEXTEST('Translation Review'!D31,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="8" t="str">
@@ -21212,6 +21337,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q32),'Translation Review'!Q32&gt;0,'Translation Review'!Q32=INT('Translation Review'!Q32)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F32" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H32="not_applicable",IFERROR(REGEXTEST('Translation Review'!D32,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="8" t="str">
@@ -21233,6 +21362,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q33),'Translation Review'!Q33&gt;0,'Translation Review'!Q33=INT('Translation Review'!Q33)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F33" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H33="not_applicable",IFERROR(REGEXTEST('Translation Review'!D33,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="8" t="str">
@@ -21254,6 +21387,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q34),'Translation Review'!Q34&gt;0,'Translation Review'!Q34=INT('Translation Review'!Q34)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F34" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H34="not_applicable",IFERROR(REGEXTEST('Translation Review'!D34,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="8" t="str">
@@ -21275,6 +21412,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q35),'Translation Review'!Q35&gt;0,'Translation Review'!Q35=INT('Translation Review'!Q35)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F35" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H35="not_applicable",IFERROR(REGEXTEST('Translation Review'!D35,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="8" t="str">
@@ -21296,6 +21437,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q36),'Translation Review'!Q36&gt;0,'Translation Review'!Q36=INT('Translation Review'!Q36)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F36" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H36="not_applicable",IFERROR(REGEXTEST('Translation Review'!D36,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="8" t="str">
@@ -21317,6 +21462,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q37),'Translation Review'!Q37&gt;0,'Translation Review'!Q37=INT('Translation Review'!Q37)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F37" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H37="not_applicable",IFERROR(REGEXTEST('Translation Review'!D37,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="8" t="str">
@@ -21338,6 +21487,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q38),'Translation Review'!Q38&gt;0,'Translation Review'!Q38=INT('Translation Review'!Q38)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F38" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H38="not_applicable",IFERROR(REGEXTEST('Translation Review'!D38,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="8" t="str">
@@ -21359,6 +21512,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q39),'Translation Review'!Q39&gt;0,'Translation Review'!Q39=INT('Translation Review'!Q39)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F39" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H39="not_applicable",IFERROR(REGEXTEST('Translation Review'!D39,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="8" t="str">
@@ -21380,6 +21537,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q40),'Translation Review'!Q40&gt;0,'Translation Review'!Q40=INT('Translation Review'!Q40)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F40" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H40="not_applicable",IFERROR(REGEXTEST('Translation Review'!D40,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="8" t="str">
@@ -21401,6 +21562,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q41),'Translation Review'!Q41&gt;0,'Translation Review'!Q41=INT('Translation Review'!Q41)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F41" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H41="not_applicable",IFERROR(REGEXTEST('Translation Review'!D41,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="8" t="str">
@@ -21422,6 +21587,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q42),'Translation Review'!Q42&gt;0,'Translation Review'!Q42=INT('Translation Review'!Q42)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F42" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H42="not_applicable",IFERROR(REGEXTEST('Translation Review'!D42,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="8" t="str">
@@ -21443,6 +21612,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q43),'Translation Review'!Q43&gt;0,'Translation Review'!Q43=INT('Translation Review'!Q43)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F43" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H43="not_applicable",IFERROR(REGEXTEST('Translation Review'!D43,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="8" t="str">
@@ -21464,6 +21637,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q44),'Translation Review'!Q44&gt;0,'Translation Review'!Q44=INT('Translation Review'!Q44)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F44" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H44="not_applicable",IFERROR(REGEXTEST('Translation Review'!D44,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="8" t="str">
@@ -21485,6 +21662,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q45),'Translation Review'!Q45&gt;0,'Translation Review'!Q45=INT('Translation Review'!Q45)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F45" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H45="not_applicable",IFERROR(REGEXTEST('Translation Review'!D45,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="8" t="str">
@@ -21506,6 +21687,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q46),'Translation Review'!Q46&gt;0,'Translation Review'!Q46=INT('Translation Review'!Q46)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F46" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H46="not_applicable",IFERROR(REGEXTEST('Translation Review'!D46,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="8" t="str">
@@ -21527,6 +21712,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q47),'Translation Review'!Q47&gt;0,'Translation Review'!Q47=INT('Translation Review'!Q47)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F47" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H47="not_applicable",IFERROR(REGEXTEST('Translation Review'!D47,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="8" t="str">
@@ -21548,6 +21737,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q48),'Translation Review'!Q48&gt;0,'Translation Review'!Q48=INT('Translation Review'!Q48)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F48" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H48="not_applicable",IFERROR(REGEXTEST('Translation Review'!D48,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="8" t="str">
@@ -21569,6 +21762,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q49),'Translation Review'!Q49&gt;0,'Translation Review'!Q49=INT('Translation Review'!Q49)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F49" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H49="not_applicable",IFERROR(REGEXTEST('Translation Review'!D49,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="8" t="str">
@@ -21590,6 +21787,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q50),'Translation Review'!Q50&gt;0,'Translation Review'!Q50=INT('Translation Review'!Q50)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F50" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H50="not_applicable",IFERROR(REGEXTEST('Translation Review'!D50,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="8" t="str">
@@ -21611,6 +21812,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q51),'Translation Review'!Q51&gt;0,'Translation Review'!Q51=INT('Translation Review'!Q51)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F51" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H51="not_applicable",IFERROR(REGEXTEST('Translation Review'!D51,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="8" t="str">
@@ -21632,6 +21837,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q52),'Translation Review'!Q52&gt;0,'Translation Review'!Q52=INT('Translation Review'!Q52)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F52" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H52="not_applicable",IFERROR(REGEXTEST('Translation Review'!D52,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="8" t="str">
@@ -21653,6 +21862,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q53),'Translation Review'!Q53&gt;0,'Translation Review'!Q53=INT('Translation Review'!Q53)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F53" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H53="not_applicable",IFERROR(REGEXTEST('Translation Review'!D53,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="8" t="str">
@@ -21674,6 +21887,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q54),'Translation Review'!Q54&gt;0,'Translation Review'!Q54=INT('Translation Review'!Q54)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F54" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H54="not_applicable",IFERROR(REGEXTEST('Translation Review'!D54,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="8" t="str">
@@ -21695,6 +21912,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q55),'Translation Review'!Q55&gt;0,'Translation Review'!Q55=INT('Translation Review'!Q55)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F55" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H55="not_applicable",IFERROR(REGEXTEST('Translation Review'!D55,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="8" t="str">
@@ -21716,6 +21937,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q56),'Translation Review'!Q56&gt;0,'Translation Review'!Q56=INT('Translation Review'!Q56)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F56" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H56="not_applicable",IFERROR(REGEXTEST('Translation Review'!D56,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="8" t="str">
@@ -21737,6 +21962,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q57),'Translation Review'!Q57&gt;0,'Translation Review'!Q57=INT('Translation Review'!Q57)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F57" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H57="not_applicable",IFERROR(REGEXTEST('Translation Review'!D57,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="8" t="str">
@@ -21758,6 +21987,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q58),'Translation Review'!Q58&gt;0,'Translation Review'!Q58=INT('Translation Review'!Q58)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F58" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H58="not_applicable",IFERROR(REGEXTEST('Translation Review'!D58,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="8" t="str">
@@ -21779,6 +22012,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q59),'Translation Review'!Q59&gt;0,'Translation Review'!Q59=INT('Translation Review'!Q59)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F59" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H59="not_applicable",IFERROR(REGEXTEST('Translation Review'!D59,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="8" t="str">
@@ -21800,6 +22037,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q60),'Translation Review'!Q60&gt;0,'Translation Review'!Q60=INT('Translation Review'!Q60)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F60" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H60="not_applicable",IFERROR(REGEXTEST('Translation Review'!D60,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="8" t="str">
@@ -21821,6 +22062,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q61),'Translation Review'!Q61&gt;0,'Translation Review'!Q61=INT('Translation Review'!Q61)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F61" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H61="not_applicable",IFERROR(REGEXTEST('Translation Review'!D61,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="8" t="str">
@@ -21842,6 +22087,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q62),'Translation Review'!Q62&gt;0,'Translation Review'!Q62=INT('Translation Review'!Q62)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F62" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H62="not_applicable",IFERROR(REGEXTEST('Translation Review'!D62,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="8" t="str">
@@ -21863,6 +22112,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q63),'Translation Review'!Q63&gt;0,'Translation Review'!Q63=INT('Translation Review'!Q63)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F63" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H63="not_applicable",IFERROR(REGEXTEST('Translation Review'!D63,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="8" t="str">
@@ -21884,6 +22137,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q64),'Translation Review'!Q64&gt;0,'Translation Review'!Q64=INT('Translation Review'!Q64)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F64" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H64="not_applicable",IFERROR(REGEXTEST('Translation Review'!D64,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="8" t="str">
@@ -21905,6 +22162,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q65),'Translation Review'!Q65&gt;0,'Translation Review'!Q65=INT('Translation Review'!Q65)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F65" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H65="not_applicable",IFERROR(REGEXTEST('Translation Review'!D65,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="8" t="str">
@@ -21926,6 +22187,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q66),'Translation Review'!Q66&gt;0,'Translation Review'!Q66=INT('Translation Review'!Q66)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F66" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H66="not_applicable",IFERROR(REGEXTEST('Translation Review'!D66,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="8" t="str">
@@ -21947,6 +22212,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q67),'Translation Review'!Q67&gt;0,'Translation Review'!Q67=INT('Translation Review'!Q67)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F67" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H67="not_applicable",IFERROR(REGEXTEST('Translation Review'!D67,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="8" t="str">
@@ -21968,6 +22237,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q68),'Translation Review'!Q68&gt;0,'Translation Review'!Q68=INT('Translation Review'!Q68)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F68" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H68="not_applicable",IFERROR(REGEXTEST('Translation Review'!D68,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="8" t="str">
@@ -21989,6 +22262,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q69),'Translation Review'!Q69&gt;0,'Translation Review'!Q69=INT('Translation Review'!Q69)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F69" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H69="not_applicable",IFERROR(REGEXTEST('Translation Review'!D69,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="8" t="str">
@@ -22010,6 +22287,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q70),'Translation Review'!Q70&gt;0,'Translation Review'!Q70=INT('Translation Review'!Q70)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F70" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H70="not_applicable",IFERROR(REGEXTEST('Translation Review'!D70,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="8" t="str">
@@ -22031,6 +22312,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q71),'Translation Review'!Q71&gt;0,'Translation Review'!Q71=INT('Translation Review'!Q71)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F71" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H71="not_applicable",IFERROR(REGEXTEST('Translation Review'!D71,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="8" t="str">
@@ -22052,6 +22337,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q72),'Translation Review'!Q72&gt;0,'Translation Review'!Q72=INT('Translation Review'!Q72)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F72" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H72="not_applicable",IFERROR(REGEXTEST('Translation Review'!D72,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="8" t="str">
@@ -22073,6 +22362,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q73),'Translation Review'!Q73&gt;0,'Translation Review'!Q73=INT('Translation Review'!Q73)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F73" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H73="not_applicable",IFERROR(REGEXTEST('Translation Review'!D73,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="8" t="str">
@@ -22094,6 +22387,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q74),'Translation Review'!Q74&gt;0,'Translation Review'!Q74=INT('Translation Review'!Q74)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F74" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H74="not_applicable",IFERROR(REGEXTEST('Translation Review'!D74,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="8" t="str">
@@ -22115,6 +22412,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q75),'Translation Review'!Q75&gt;0,'Translation Review'!Q75=INT('Translation Review'!Q75)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F75" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H75="not_applicable",IFERROR(REGEXTEST('Translation Review'!D75,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="8" t="str">
@@ -22136,6 +22437,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q76),'Translation Review'!Q76&gt;0,'Translation Review'!Q76=INT('Translation Review'!Q76)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F76" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H76="not_applicable",IFERROR(REGEXTEST('Translation Review'!D76,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="8" t="str">
@@ -22157,6 +22462,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q77),'Translation Review'!Q77&gt;0,'Translation Review'!Q77=INT('Translation Review'!Q77)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F77" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H77="not_applicable",IFERROR(REGEXTEST('Translation Review'!D77,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="8" t="str">
@@ -22178,6 +22487,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q78),'Translation Review'!Q78&gt;0,'Translation Review'!Q78=INT('Translation Review'!Q78)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F78" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H78="not_applicable",IFERROR(REGEXTEST('Translation Review'!D78,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="8" t="str">
@@ -22199,6 +22512,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q79),'Translation Review'!Q79&gt;0,'Translation Review'!Q79=INT('Translation Review'!Q79)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F79" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H79="not_applicable",IFERROR(REGEXTEST('Translation Review'!D79,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="8" t="str">
@@ -22220,6 +22537,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q80),'Translation Review'!Q80&gt;0,'Translation Review'!Q80=INT('Translation Review'!Q80)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F80" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H80="not_applicable",IFERROR(REGEXTEST('Translation Review'!D80,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="8" t="str">
@@ -22241,6 +22562,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q81),'Translation Review'!Q81&gt;0,'Translation Review'!Q81=INT('Translation Review'!Q81)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F81" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H81="not_applicable",IFERROR(REGEXTEST('Translation Review'!D81,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="8" t="str">
@@ -22262,6 +22587,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q82),'Translation Review'!Q82&gt;0,'Translation Review'!Q82=INT('Translation Review'!Q82)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F82" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H82="not_applicable",IFERROR(REGEXTEST('Translation Review'!D82,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="8" t="str">
@@ -22283,6 +22612,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q83),'Translation Review'!Q83&gt;0,'Translation Review'!Q83=INT('Translation Review'!Q83)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F83" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H83="not_applicable",IFERROR(REGEXTEST('Translation Review'!D83,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="8" t="str">
@@ -22304,6 +22637,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q84),'Translation Review'!Q84&gt;0,'Translation Review'!Q84=INT('Translation Review'!Q84)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F84" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H84="not_applicable",IFERROR(REGEXTEST('Translation Review'!D84,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="8" t="str">
@@ -22325,6 +22662,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q85),'Translation Review'!Q85&gt;0,'Translation Review'!Q85=INT('Translation Review'!Q85)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F85" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H85="not_applicable",IFERROR(REGEXTEST('Translation Review'!D85,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="8" t="str">
@@ -22346,6 +22687,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q86),'Translation Review'!Q86&gt;0,'Translation Review'!Q86=INT('Translation Review'!Q86)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F86" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H86="not_applicable",IFERROR(REGEXTEST('Translation Review'!D86,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="8" t="str">
@@ -22367,6 +22712,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q87),'Translation Review'!Q87&gt;0,'Translation Review'!Q87=INT('Translation Review'!Q87)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F87" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H87="not_applicable",IFERROR(REGEXTEST('Translation Review'!D87,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="8" t="str">
@@ -22388,6 +22737,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q88),'Translation Review'!Q88&gt;0,'Translation Review'!Q88=INT('Translation Review'!Q88)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F88" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H88="not_applicable",IFERROR(REGEXTEST('Translation Review'!D88,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="8" t="str">
@@ -22409,6 +22762,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q89),'Translation Review'!Q89&gt;0,'Translation Review'!Q89=INT('Translation Review'!Q89)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F89" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H89="not_applicable",IFERROR(REGEXTEST('Translation Review'!D89,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="8" t="str">
@@ -22430,6 +22787,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q90),'Translation Review'!Q90&gt;0,'Translation Review'!Q90=INT('Translation Review'!Q90)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F90" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H90="not_applicable",IFERROR(REGEXTEST('Translation Review'!D90,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="8" t="str">
@@ -22451,6 +22812,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q91),'Translation Review'!Q91&gt;0,'Translation Review'!Q91=INT('Translation Review'!Q91)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F91" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H91="not_applicable",IFERROR(REGEXTEST('Translation Review'!D91,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="8" t="str">
@@ -22472,6 +22837,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q92),'Translation Review'!Q92&gt;0,'Translation Review'!Q92=INT('Translation Review'!Q92)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F92" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H92="not_applicable",IFERROR(REGEXTEST('Translation Review'!D92,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="8" t="str">
@@ -22493,6 +22862,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q93),'Translation Review'!Q93&gt;0,'Translation Review'!Q93=INT('Translation Review'!Q93)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F93" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H93="not_applicable",IFERROR(REGEXTEST('Translation Review'!D93,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="8" t="str">
@@ -22514,6 +22887,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q94),'Translation Review'!Q94&gt;0,'Translation Review'!Q94=INT('Translation Review'!Q94)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F94" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H94="not_applicable",IFERROR(REGEXTEST('Translation Review'!D94,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="8" t="str">
@@ -22535,6 +22912,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q95),'Translation Review'!Q95&gt;0,'Translation Review'!Q95=INT('Translation Review'!Q95)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F95" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H95="not_applicable",IFERROR(REGEXTEST('Translation Review'!D95,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="8" t="str">
@@ -22556,6 +22937,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q96),'Translation Review'!Q96&gt;0,'Translation Review'!Q96=INT('Translation Review'!Q96)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F96" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H96="not_applicable",IFERROR(REGEXTEST('Translation Review'!D96,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="8" t="str">
@@ -22577,6 +22962,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q97),'Translation Review'!Q97&gt;0,'Translation Review'!Q97=INT('Translation Review'!Q97)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F97" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H97="not_applicable",IFERROR(REGEXTEST('Translation Review'!D97,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="8" t="str">
@@ -22598,6 +22987,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q98),'Translation Review'!Q98&gt;0,'Translation Review'!Q98=INT('Translation Review'!Q98)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F98" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H98="not_applicable",IFERROR(REGEXTEST('Translation Review'!D98,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="8" t="str">
@@ -22619,6 +23012,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q99),'Translation Review'!Q99&gt;0,'Translation Review'!Q99=INT('Translation Review'!Q99)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F99" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H99="not_applicable",IFERROR(REGEXTEST('Translation Review'!D99,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="8" t="str">
@@ -22640,6 +23037,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q100),'Translation Review'!Q100&gt;0,'Translation Review'!Q100=INT('Translation Review'!Q100)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F100" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H100="not_applicable",IFERROR(REGEXTEST('Translation Review'!D100,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="8" t="str">
@@ -22661,6 +23062,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q101),'Translation Review'!Q101&gt;0,'Translation Review'!Q101=INT('Translation Review'!Q101)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F101" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H101="not_applicable",IFERROR(REGEXTEST('Translation Review'!D101,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
       <x:c r="A102" s="8" t="str">
@@ -22682,6 +23087,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q102),'Translation Review'!Q102&gt;0,'Translation Review'!Q102=INT('Translation Review'!Q102)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F102" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H102="not_applicable",IFERROR(REGEXTEST('Translation Review'!D102,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
       <x:c r="A103" s="8" t="str">
@@ -22703,6 +23112,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q103),'Translation Review'!Q103&gt;0,'Translation Review'!Q103=INT('Translation Review'!Q103)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F103" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H103="not_applicable",IFERROR(REGEXTEST('Translation Review'!D103,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
       <x:c r="A104" s="8" t="str">
@@ -22724,6 +23137,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q104),'Translation Review'!Q104&gt;0,'Translation Review'!Q104=INT('Translation Review'!Q104)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F104" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H104="not_applicable",IFERROR(REGEXTEST('Translation Review'!D104,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="24" customHeight="1">
       <x:c r="A105" s="8" t="str">
@@ -22745,6 +23162,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q105),'Translation Review'!Q105&gt;0,'Translation Review'!Q105=INT('Translation Review'!Q105)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F105" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H105="not_applicable",IFERROR(REGEXTEST('Translation Review'!D105,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="24" customHeight="1">
       <x:c r="A106" s="8" t="str">
@@ -22766,6 +23187,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q106),'Translation Review'!Q106&gt;0,'Translation Review'!Q106=INT('Translation Review'!Q106)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F106" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H106="not_applicable",IFERROR(REGEXTEST('Translation Review'!D106,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="24" customHeight="1">
       <x:c r="A107" s="8" t="str">
@@ -22787,6 +23212,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q107),'Translation Review'!Q107&gt;0,'Translation Review'!Q107=INT('Translation Review'!Q107)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F107" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H107="not_applicable",IFERROR(REGEXTEST('Translation Review'!D107,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="24" customHeight="1">
       <x:c r="A108" s="8" t="str">
@@ -22808,6 +23237,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q108),'Translation Review'!Q108&gt;0,'Translation Review'!Q108=INT('Translation Review'!Q108)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F108" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H108="not_applicable",IFERROR(REGEXTEST('Translation Review'!D108,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="24" customHeight="1">
       <x:c r="A109" s="8" t="str">
@@ -22829,6 +23262,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q109),'Translation Review'!Q109&gt;0,'Translation Review'!Q109=INT('Translation Review'!Q109)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F109" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H109="not_applicable",IFERROR(REGEXTEST('Translation Review'!D109,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="24" customHeight="1">
       <x:c r="A110" s="8" t="str">
@@ -22850,6 +23287,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q110),'Translation Review'!Q110&gt;0,'Translation Review'!Q110=INT('Translation Review'!Q110)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F110" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H110="not_applicable",IFERROR(REGEXTEST('Translation Review'!D110,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="24" customHeight="1">
       <x:c r="A111" s="8" t="str">
@@ -22871,6 +23312,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q111),'Translation Review'!Q111&gt;0,'Translation Review'!Q111=INT('Translation Review'!Q111)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F111" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H111="not_applicable",IFERROR(REGEXTEST('Translation Review'!D111,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="24" customHeight="1">
       <x:c r="A112" s="8" t="str">
@@ -22892,6 +23337,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q112),'Translation Review'!Q112&gt;0,'Translation Review'!Q112=INT('Translation Review'!Q112)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F112" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H112="not_applicable",IFERROR(REGEXTEST('Translation Review'!D112,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="24" customHeight="1">
       <x:c r="A113" s="8" t="str">
@@ -22913,6 +23362,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q113),'Translation Review'!Q113&gt;0,'Translation Review'!Q113=INT('Translation Review'!Q113)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F113" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H113="not_applicable",IFERROR(REGEXTEST('Translation Review'!D113,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="24" customHeight="1">
       <x:c r="A114" s="8" t="str">
@@ -22934,6 +23387,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q114),'Translation Review'!Q114&gt;0,'Translation Review'!Q114=INT('Translation Review'!Q114)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F114" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H114="not_applicable",IFERROR(REGEXTEST('Translation Review'!D114,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="24" customHeight="1">
       <x:c r="A115" s="8" t="str">
@@ -22955,6 +23412,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q115),'Translation Review'!Q115&gt;0,'Translation Review'!Q115=INT('Translation Review'!Q115)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F115" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H115="not_applicable",IFERROR(REGEXTEST('Translation Review'!D115,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="24" customHeight="1">
       <x:c r="A116" s="8" t="str">
@@ -22976,6 +23437,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q116),'Translation Review'!Q116&gt;0,'Translation Review'!Q116=INT('Translation Review'!Q116)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F116" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H116="not_applicable",IFERROR(REGEXTEST('Translation Review'!D116,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="24" customHeight="1">
       <x:c r="A117" s="8" t="str">
@@ -22997,6 +23462,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q117),'Translation Review'!Q117&gt;0,'Translation Review'!Q117=INT('Translation Review'!Q117)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F117" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H117="not_applicable",IFERROR(REGEXTEST('Translation Review'!D117,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="24" customHeight="1">
       <x:c r="A118" s="8" t="str">
@@ -23018,6 +23487,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q118),'Translation Review'!Q118&gt;0,'Translation Review'!Q118=INT('Translation Review'!Q118)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F118" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H118="not_applicable",IFERROR(REGEXTEST('Translation Review'!D118,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="24" customHeight="1">
       <x:c r="A119" s="8" t="str">
@@ -23039,6 +23512,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q119),'Translation Review'!Q119&gt;0,'Translation Review'!Q119=INT('Translation Review'!Q119)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F119" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H119="not_applicable",IFERROR(REGEXTEST('Translation Review'!D119,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="24" customHeight="1">
       <x:c r="A120" s="8" t="str">
@@ -23060,6 +23537,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q120),'Translation Review'!Q120&gt;0,'Translation Review'!Q120=INT('Translation Review'!Q120)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F120" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H120="not_applicable",IFERROR(REGEXTEST('Translation Review'!D120,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="24" customHeight="1">
       <x:c r="A121" s="8" t="str">
@@ -23081,6 +23562,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q121),'Translation Review'!Q121&gt;0,'Translation Review'!Q121=INT('Translation Review'!Q121)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F121" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H121="not_applicable",IFERROR(REGEXTEST('Translation Review'!D121,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="24" customHeight="1">
       <x:c r="A122" s="8" t="str">
@@ -23102,6 +23587,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q122),'Translation Review'!Q122&gt;0,'Translation Review'!Q122=INT('Translation Review'!Q122)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F122" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H122="not_applicable",IFERROR(REGEXTEST('Translation Review'!D122,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="24" customHeight="1">
       <x:c r="A123" s="8" t="str">
@@ -23123,6 +23612,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q123),'Translation Review'!Q123&gt;0,'Translation Review'!Q123=INT('Translation Review'!Q123)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F123" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H123="not_applicable",IFERROR(REGEXTEST('Translation Review'!D123,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="24" customHeight="1">
       <x:c r="A124" s="8" t="str">
@@ -23144,6 +23637,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q124),'Translation Review'!Q124&gt;0,'Translation Review'!Q124=INT('Translation Review'!Q124)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F124" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H124="not_applicable",IFERROR(REGEXTEST('Translation Review'!D124,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="24" customHeight="1">
       <x:c r="A125" s="8" t="str">
@@ -23165,6 +23662,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q125),'Translation Review'!Q125&gt;0,'Translation Review'!Q125=INT('Translation Review'!Q125)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F125" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H125="not_applicable",IFERROR(REGEXTEST('Translation Review'!D125,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="24" customHeight="1">
       <x:c r="A126" s="8" t="str">
@@ -23186,6 +23687,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q126),'Translation Review'!Q126&gt;0,'Translation Review'!Q126=INT('Translation Review'!Q126)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F126" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H126="not_applicable",IFERROR(REGEXTEST('Translation Review'!D126,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="24" customHeight="1">
       <x:c r="A127" s="8" t="str">
@@ -23207,6 +23712,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q127),'Translation Review'!Q127&gt;0,'Translation Review'!Q127=INT('Translation Review'!Q127)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F127" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H127="not_applicable",IFERROR(REGEXTEST('Translation Review'!D127,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="24" customHeight="1">
       <x:c r="A128" s="8" t="str">
@@ -23228,6 +23737,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q128),'Translation Review'!Q128&gt;0,'Translation Review'!Q128=INT('Translation Review'!Q128)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F128" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H128="not_applicable",IFERROR(REGEXTEST('Translation Review'!D128,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="129" ht="24" customHeight="1">
       <x:c r="A129" s="8" t="str">
@@ -23249,6 +23762,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q129),'Translation Review'!Q129&gt;0,'Translation Review'!Q129=INT('Translation Review'!Q129)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F129" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H129="not_applicable",IFERROR(REGEXTEST('Translation Review'!D129,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="130" ht="24" customHeight="1">
       <x:c r="A130" s="8" t="str">
@@ -23270,6 +23787,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q130),'Translation Review'!Q130&gt;0,'Translation Review'!Q130=INT('Translation Review'!Q130)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F130" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H130="not_applicable",IFERROR(REGEXTEST('Translation Review'!D130,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="131" ht="24" customHeight="1">
       <x:c r="A131" s="8" t="str">
@@ -23291,6 +23812,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q131),'Translation Review'!Q131&gt;0,'Translation Review'!Q131=INT('Translation Review'!Q131)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F131" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H131="not_applicable",IFERROR(REGEXTEST('Translation Review'!D131,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="132" ht="24" customHeight="1">
       <x:c r="A132" s="8" t="str">
@@ -23312,6 +23837,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q132),'Translation Review'!Q132&gt;0,'Translation Review'!Q132=INT('Translation Review'!Q132)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F132" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H132="not_applicable",IFERROR(REGEXTEST('Translation Review'!D132,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="133" ht="24" customHeight="1">
       <x:c r="A133" s="8" t="str">
@@ -23333,6 +23862,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q133),'Translation Review'!Q133&gt;0,'Translation Review'!Q133=INT('Translation Review'!Q133)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F133" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H133="not_applicable",IFERROR(REGEXTEST('Translation Review'!D133,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="24" customHeight="1">
       <x:c r="A134" s="8" t="str">
@@ -23354,6 +23887,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q134),'Translation Review'!Q134&gt;0,'Translation Review'!Q134=INT('Translation Review'!Q134)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F134" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H134="not_applicable",IFERROR(REGEXTEST('Translation Review'!D134,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="24" customHeight="1">
       <x:c r="A135" s="8" t="str">
@@ -23375,6 +23912,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q135),'Translation Review'!Q135&gt;0,'Translation Review'!Q135=INT('Translation Review'!Q135)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F135" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H135="not_applicable",IFERROR(REGEXTEST('Translation Review'!D135,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="136" ht="24" customHeight="1">
       <x:c r="A136" s="8" t="str">
@@ -23396,6 +23937,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q136),'Translation Review'!Q136&gt;0,'Translation Review'!Q136=INT('Translation Review'!Q136)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F136" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H136="not_applicable",IFERROR(REGEXTEST('Translation Review'!D136,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="137" ht="24" customHeight="1">
       <x:c r="A137" s="8" t="str">
@@ -23417,6 +23962,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q137),'Translation Review'!Q137&gt;0,'Translation Review'!Q137=INT('Translation Review'!Q137)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F137" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H137="not_applicable",IFERROR(REGEXTEST('Translation Review'!D137,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="24" customHeight="1">
       <x:c r="A138" s="8" t="str">
@@ -23438,6 +23987,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q138),'Translation Review'!Q138&gt;0,'Translation Review'!Q138=INT('Translation Review'!Q138)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F138" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H138="not_applicable",IFERROR(REGEXTEST('Translation Review'!D138,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="24" customHeight="1">
       <x:c r="A139" s="8" t="str">
@@ -23459,6 +24012,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q139),'Translation Review'!Q139&gt;0,'Translation Review'!Q139=INT('Translation Review'!Q139)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F139" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H139="not_applicable",IFERROR(REGEXTEST('Translation Review'!D139,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="140" ht="24" customHeight="1">
       <x:c r="A140" s="8" t="str">
@@ -23480,6 +24037,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q140),'Translation Review'!Q140&gt;0,'Translation Review'!Q140=INT('Translation Review'!Q140)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F140" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H140="not_applicable",IFERROR(REGEXTEST('Translation Review'!D140,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="24" customHeight="1">
       <x:c r="A141" s="8" t="str">
@@ -23501,6 +24062,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q141),'Translation Review'!Q141&gt;0,'Translation Review'!Q141=INT('Translation Review'!Q141)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F141" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H141="not_applicable",IFERROR(REGEXTEST('Translation Review'!D141,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="24" customHeight="1">
       <x:c r="A142" s="8" t="str">
@@ -23522,6 +24087,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q142),'Translation Review'!Q142&gt;0,'Translation Review'!Q142=INT('Translation Review'!Q142)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F142" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H142="not_applicable",IFERROR(REGEXTEST('Translation Review'!D142,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="143" ht="24" customHeight="1">
       <x:c r="A143" s="8" t="str">
@@ -23543,6 +24112,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q143),'Translation Review'!Q143&gt;0,'Translation Review'!Q143=INT('Translation Review'!Q143)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F143" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H143="not_applicable",IFERROR(REGEXTEST('Translation Review'!D143,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="144" ht="24" customHeight="1">
       <x:c r="A144" s="8" t="str">
@@ -23564,6 +24137,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q144),'Translation Review'!Q144&gt;0,'Translation Review'!Q144=INT('Translation Review'!Q144)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F144" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H144="not_applicable",IFERROR(REGEXTEST('Translation Review'!D144,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="145" ht="24" customHeight="1">
       <x:c r="A145" s="8" t="str">
@@ -23585,6 +24162,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q145),'Translation Review'!Q145&gt;0,'Translation Review'!Q145=INT('Translation Review'!Q145)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F145" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H145="not_applicable",IFERROR(REGEXTEST('Translation Review'!D145,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="146" ht="24" customHeight="1">
       <x:c r="A146" s="8" t="str">
@@ -23606,6 +24187,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q146),'Translation Review'!Q146&gt;0,'Translation Review'!Q146=INT('Translation Review'!Q146)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F146" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H146="not_applicable",IFERROR(REGEXTEST('Translation Review'!D146,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="147" ht="24" customHeight="1">
       <x:c r="A147" s="8" t="str">
@@ -23627,6 +24212,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q147),'Translation Review'!Q147&gt;0,'Translation Review'!Q147=INT('Translation Review'!Q147)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F147" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H147="not_applicable",IFERROR(REGEXTEST('Translation Review'!D147,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="148" ht="24" customHeight="1">
       <x:c r="A148" s="8" t="str">
@@ -23648,6 +24237,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q148),'Translation Review'!Q148&gt;0,'Translation Review'!Q148=INT('Translation Review'!Q148)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F148" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H148="not_applicable",IFERROR(REGEXTEST('Translation Review'!D148,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="24" customHeight="1">
       <x:c r="A149" s="8" t="str">
@@ -23669,6 +24262,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q149),'Translation Review'!Q149&gt;0,'Translation Review'!Q149=INT('Translation Review'!Q149)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F149" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H149="not_applicable",IFERROR(REGEXTEST('Translation Review'!D149,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="24" customHeight="1">
       <x:c r="A150" s="8" t="str">
@@ -23690,6 +24287,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q150),'Translation Review'!Q150&gt;0,'Translation Review'!Q150=INT('Translation Review'!Q150)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F150" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H150="not_applicable",IFERROR(REGEXTEST('Translation Review'!D150,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="24" customHeight="1">
       <x:c r="A151" s="8" t="str">
@@ -23711,6 +24312,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q151),'Translation Review'!Q151&gt;0,'Translation Review'!Q151=INT('Translation Review'!Q151)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F151" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H151="not_applicable",IFERROR(REGEXTEST('Translation Review'!D151,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="24" customHeight="1">
       <x:c r="A152" s="8" t="str">
@@ -23732,6 +24337,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q152),'Translation Review'!Q152&gt;0,'Translation Review'!Q152=INT('Translation Review'!Q152)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F152" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H152="not_applicable",IFERROR(REGEXTEST('Translation Review'!D152,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="24" customHeight="1">
       <x:c r="A153" s="8" t="str">
@@ -23753,6 +24362,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q153),'Translation Review'!Q153&gt;0,'Translation Review'!Q153=INT('Translation Review'!Q153)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F153" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H153="not_applicable",IFERROR(REGEXTEST('Translation Review'!D153,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="24" customHeight="1">
       <x:c r="A154" s="8" t="str">
@@ -23774,6 +24387,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q154),'Translation Review'!Q154&gt;0,'Translation Review'!Q154=INT('Translation Review'!Q154)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F154" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H154="not_applicable",IFERROR(REGEXTEST('Translation Review'!D154,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="24" customHeight="1">
       <x:c r="A155" s="8" t="str">
@@ -23795,6 +24412,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q155),'Translation Review'!Q155&gt;0,'Translation Review'!Q155=INT('Translation Review'!Q155)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F155" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H155="not_applicable",IFERROR(REGEXTEST('Translation Review'!D155,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="24" customHeight="1">
       <x:c r="A156" s="8" t="str">
@@ -23816,6 +24437,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q156),'Translation Review'!Q156&gt;0,'Translation Review'!Q156=INT('Translation Review'!Q156)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F156" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H156="not_applicable",IFERROR(REGEXTEST('Translation Review'!D156,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="157" ht="24" customHeight="1">
       <x:c r="A157" s="8" t="str">
@@ -23837,6 +24462,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q157),'Translation Review'!Q157&gt;0,'Translation Review'!Q157=INT('Translation Review'!Q157)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F157" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H157="not_applicable",IFERROR(REGEXTEST('Translation Review'!D157,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="24" customHeight="1">
       <x:c r="A158" s="8" t="str">
@@ -23858,6 +24487,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q158),'Translation Review'!Q158&gt;0,'Translation Review'!Q158=INT('Translation Review'!Q158)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F158" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H158="not_applicable",IFERROR(REGEXTEST('Translation Review'!D158,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="24" customHeight="1">
       <x:c r="A159" s="8" t="str">
@@ -23879,6 +24512,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q159),'Translation Review'!Q159&gt;0,'Translation Review'!Q159=INT('Translation Review'!Q159)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F159" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H159="not_applicable",IFERROR(REGEXTEST('Translation Review'!D159,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="24" customHeight="1">
       <x:c r="A160" s="8" t="str">
@@ -23900,6 +24537,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q160),'Translation Review'!Q160&gt;0,'Translation Review'!Q160=INT('Translation Review'!Q160)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F160" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H160="not_applicable",IFERROR(REGEXTEST('Translation Review'!D160,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="24" customHeight="1">
       <x:c r="A161" s="8" t="str">
@@ -23921,6 +24562,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q161),'Translation Review'!Q161&gt;0,'Translation Review'!Q161=INT('Translation Review'!Q161)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F161" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H161="not_applicable",IFERROR(REGEXTEST('Translation Review'!D161,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="24" customHeight="1">
       <x:c r="A162" s="8" t="str">
@@ -23942,6 +24587,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q162),'Translation Review'!Q162&gt;0,'Translation Review'!Q162=INT('Translation Review'!Q162)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F162" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H162="not_applicable",IFERROR(REGEXTEST('Translation Review'!D162,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="24" customHeight="1">
       <x:c r="A163" s="8" t="str">
@@ -23963,6 +24612,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q163),'Translation Review'!Q163&gt;0,'Translation Review'!Q163=INT('Translation Review'!Q163)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F163" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H163="not_applicable",IFERROR(REGEXTEST('Translation Review'!D163,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="24" customHeight="1">
       <x:c r="A164" s="8" t="str">
@@ -23984,6 +24637,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q164),'Translation Review'!Q164&gt;0,'Translation Review'!Q164=INT('Translation Review'!Q164)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F164" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H164="not_applicable",IFERROR(REGEXTEST('Translation Review'!D164,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="24" customHeight="1">
       <x:c r="A165" s="8" t="str">
@@ -24005,6 +24662,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q165),'Translation Review'!Q165&gt;0,'Translation Review'!Q165=INT('Translation Review'!Q165)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F165" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H165="not_applicable",IFERROR(REGEXTEST('Translation Review'!D165,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="24" customHeight="1">
       <x:c r="A166" s="8" t="str">
@@ -24026,6 +24687,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q166),'Translation Review'!Q166&gt;0,'Translation Review'!Q166=INT('Translation Review'!Q166)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F166" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H166="not_applicable",IFERROR(REGEXTEST('Translation Review'!D166,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="24" customHeight="1">
       <x:c r="A167" s="8" t="str">
@@ -24047,6 +24712,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q167),'Translation Review'!Q167&gt;0,'Translation Review'!Q167=INT('Translation Review'!Q167)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F167" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H167="not_applicable",IFERROR(REGEXTEST('Translation Review'!D167,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="168" ht="24" customHeight="1">
       <x:c r="A168" s="8" t="str">
@@ -24068,6 +24737,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q168),'Translation Review'!Q168&gt;0,'Translation Review'!Q168=INT('Translation Review'!Q168)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F168" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H168="not_applicable",IFERROR(REGEXTEST('Translation Review'!D168,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="169" ht="24" customHeight="1">
       <x:c r="A169" s="8" t="str">
@@ -24089,6 +24762,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q169),'Translation Review'!Q169&gt;0,'Translation Review'!Q169=INT('Translation Review'!Q169)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F169" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H169="not_applicable",IFERROR(REGEXTEST('Translation Review'!D169,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="170" ht="24" customHeight="1">
       <x:c r="A170" s="8" t="str">
@@ -24110,6 +24787,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q170),'Translation Review'!Q170&gt;0,'Translation Review'!Q170=INT('Translation Review'!Q170)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F170" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H170="not_applicable",IFERROR(REGEXTEST('Translation Review'!D170,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="171" ht="24" customHeight="1">
       <x:c r="A171" s="8" t="str">
@@ -24131,6 +24812,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q171),'Translation Review'!Q171&gt;0,'Translation Review'!Q171=INT('Translation Review'!Q171)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F171" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H171="not_applicable",IFERROR(REGEXTEST('Translation Review'!D171,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="172" ht="24" customHeight="1">
       <x:c r="A172" s="8" t="str">
@@ -24152,6 +24837,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q172),'Translation Review'!Q172&gt;0,'Translation Review'!Q172=INT('Translation Review'!Q172)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F172" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H172="not_applicable",IFERROR(REGEXTEST('Translation Review'!D172,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="173" ht="24" customHeight="1">
       <x:c r="A173" s="8" t="str">
@@ -24173,6 +24862,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q173),'Translation Review'!Q173&gt;0,'Translation Review'!Q173=INT('Translation Review'!Q173)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F173" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H173="not_applicable",IFERROR(REGEXTEST('Translation Review'!D173,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="24" customHeight="1">
       <x:c r="A174" s="8" t="str">
@@ -24194,6 +24887,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q174),'Translation Review'!Q174&gt;0,'Translation Review'!Q174=INT('Translation Review'!Q174)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F174" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H174="not_applicable",IFERROR(REGEXTEST('Translation Review'!D174,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="175" ht="24" customHeight="1">
       <x:c r="A175" s="8" t="str">
@@ -24215,6 +24912,10 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q175),'Translation Review'!Q175&gt;0,'Translation Review'!Q175=INT('Translation Review'!Q175)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F175" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H175="not_applicable",IFERROR(REGEXTEST('Translation Review'!D175,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="176" ht="24" customHeight="1">
       <x:c r="A176" s="8" t="str">
@@ -24236,16 +24937,20 @@
         <x:f>IF(AND(ISNUMBER('Translation Review'!Q176),'Translation Review'!Q176&gt;0,'Translation Review'!Q176=INT('Translation Review'!Q176)),0,1)</x:f>
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F176" s="8" t="n">
+        <x:f>IF(AND('Translation Review'!H176="not_applicable",IFERROR(REGEXTEST('Translation Review'!D176,"(?:\d+\s*(?:กก\.?|กิโลกรัม|ซม\.?|เมตร|นาที|ปี|คน)|ชั่วโมง)"),TRUE)),1,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="B2:E176">
+  <x:conditionalFormatting sqref="B2:F176">
     <x:cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57071b6ffe424727"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc5c41e470724f13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24403,7 +25108,7 @@
         <x:v>Unresolved or invalid review checks</x:v>
       </x:c>
       <x:c r="B18" s="21" t="n">
-        <x:f>COUNTIF('Translation Review'!G2:G176,"&lt;&gt;pass")+COUNTIFS('Translation Review'!H2:H176,"&lt;&gt;pass",'Translation Review'!H2:H176,"&lt;&gt;not_applicable")+COUNTIF('Translation Review'!I2:I176,"&lt;&gt;pass")+COUNTIF('Translation Review'!J2:J176,"&lt;&gt;pass")+COUNTIF('Translation Review'!K2:K176,"&lt;&gt;pass")+COUNTIF('Translation Review'!L2:L176,"&lt;&gt;pass")</x:f>
+        <x:f>COUNTIF('Translation Review'!G2:G176,"&lt;&gt;pass")+COUNTIFS('Translation Review'!H2:H176,"&lt;&gt;pass",'Translation Review'!H2:H176,"&lt;&gt;not_applicable")+COUNTIF('Translation Review'!I2:I176,"&lt;&gt;pass")+COUNTIF('Translation Review'!J2:J176,"&lt;&gt;pass")+COUNTIF('Translation Review'!K2:K176,"&lt;&gt;pass")+COUNTIF('Translation Review'!L2:L176,"&lt;&gt;pass")+SUM('Gate Audit'!F2:F176)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>